<commit_message>
added additional rules + documentation
</commit_message>
<xml_diff>
--- a/sample.xlsx
+++ b/sample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\kelvin\python\infinito\template-writer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C433F33F-7120-47AC-BEBB-881711EC1E21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9A9A32F-1DAE-4841-83CF-FC895EF6FFEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" xr2:uid="{59884333-ABBA-4849-8D19-5D06745C2A80}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="21">
   <si>
     <t>a</t>
   </si>
@@ -70,6 +70,24 @@
   </si>
   <si>
     <t>s</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>b</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>d</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>someValue</t>
   </si>
 </sst>
 </file>
@@ -421,15 +439,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA9C3A17-E802-4849-8E8E-3D620C289BE3}">
-  <dimension ref="G1:LA294"/>
+  <dimension ref="C1:LA294"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="7:313" x14ac:dyDescent="0.25">
+    <row r="1" spans="3:313" x14ac:dyDescent="0.25">
       <c r="LA1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="7:313" x14ac:dyDescent="0.25">
+    <row r="9" spans="3:313" x14ac:dyDescent="0.25">
       <c r="G9" t="s">
         <v>1</v>
       </c>
@@ -446,7 +464,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="7:313" x14ac:dyDescent="0.25">
+    <row r="10" spans="3:313" x14ac:dyDescent="0.25">
       <c r="G10">
         <v>1</v>
       </c>
@@ -463,7 +481,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="7:313" x14ac:dyDescent="0.25">
+    <row r="11" spans="3:313" x14ac:dyDescent="0.25">
       <c r="G11">
         <v>2</v>
       </c>
@@ -480,7 +498,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="7:313" x14ac:dyDescent="0.25">
+    <row r="12" spans="3:313" x14ac:dyDescent="0.25">
       <c r="G12">
         <v>3</v>
       </c>
@@ -497,7 +515,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="7:313" x14ac:dyDescent="0.25">
+    <row r="13" spans="3:313" x14ac:dyDescent="0.25">
       <c r="G13">
         <v>4</v>
       </c>
@@ -509,6 +527,91 @@
       </c>
       <c r="K13" t="s">
         <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="3:313" x14ac:dyDescent="0.25">
+      <c r="C16" t="s">
+        <v>1</v>
+      </c>
+      <c r="D16" t="s">
+        <v>3</v>
+      </c>
+      <c r="E16" t="s">
+        <v>4</v>
+      </c>
+      <c r="F16" t="s">
+        <v>5</v>
+      </c>
+      <c r="G16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17" t="s">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>0</v>
+      </c>
+      <c r="F17" t="s">
+        <v>0</v>
+      </c>
+      <c r="G17" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C18">
+        <v>2</v>
+      </c>
+      <c r="D18" t="s">
+        <v>16</v>
+      </c>
+      <c r="E18" t="s">
+        <v>17</v>
+      </c>
+      <c r="F18" t="s">
+        <v>18</v>
+      </c>
+      <c r="G18" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C19">
+        <v>3</v>
+      </c>
+      <c r="D19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E19" t="s">
+        <v>18</v>
+      </c>
+      <c r="F19" t="s">
+        <v>17</v>
+      </c>
+      <c r="G19" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C21" t="s">
+        <v>20</v>
+      </c>
+      <c r="D21" t="s">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s">
+        <v>16</v>
+      </c>
+      <c r="F21" t="s">
+        <v>17</v>
+      </c>
+      <c r="G21" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="294" spans="15:15" x14ac:dyDescent="0.25">

</xml_diff>